<commit_message>
refactor: introduce `ExportType` enum and `DocumentExportStrategy` for improved type clarity and strategy reusability
</commit_message>
<xml_diff>
--- a/tw-core/src/test/resources/dev.hertlein.timesheetwizard.core.exporting.domain.service.strategy/timesheet_v1_PiedPiper_20220101-20221231.xlsx
+++ b/tw-core/src/test/resources/dev.hertlein.timesheetwizard.core.exporting.domain.service.strategy/timesheet_v1_PiedPiper_20220101-20221231.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11116"/>
   <workbookPr showInkAnnotation="0" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tino/IdeaProjects/timesheet-wizard-2/tw-app/src/test/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tino/IdeaProjects/timesheet-wizard/tw-core/src/test/resources/dev.hertlein.timesheetwizard.core.exporting.domain.service.strategy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1464C7FC-87E9-1D47-B4F9-326E9CACCEFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EA37E98-70CB-3F41-B383-FE0878BFCB13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -79,13 +79,13 @@
     <t>a-contact-email</t>
   </si>
   <si>
-    <t>a-project</t>
-  </si>
-  <si>
     <t>a-task</t>
   </si>
   <si>
     <t>a-tag</t>
+  </si>
+  <si>
+    <t>a-project-name</t>
   </si>
 </sst>
 </file>
@@ -1201,13 +1201,13 @@
         <v>44562</v>
       </c>
       <c r="B7" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>12</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>13</v>
       </c>
       <c r="E7" s="9">
         <v>2</v>

</xml_diff>

<commit_message>
feat: replace `task` with `task` and `description` fields in timesheet export and update grouping logic
</commit_message>
<xml_diff>
--- a/tw-core/src/test/resources/dev.hertlein.timesheetwizard.core.exporting.domain.service.strategy/timesheet_v1_PiedPiper_20220101-20221231.xlsx
+++ b/tw-core/src/test/resources/dev.hertlein.timesheetwizard.core.exporting.domain.service.strategy/timesheet_v1_PiedPiper_20220101-20221231.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tino/IdeaProjects/timesheet-wizard/tw-core/src/test/resources/dev.hertlein.timesheetwizard.core.exporting.domain.service.strategy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EA37E98-70CB-3F41-B383-FE0878BFCB13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49E6A959-9FD1-1949-93B7-3C32B469B823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Timesheet!$6:$6</definedName>
     <definedName name="WorkweekHours">Timesheet!#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -79,13 +79,13 @@
     <t>a-contact-email</t>
   </si>
   <si>
-    <t>a-task</t>
-  </si>
-  <si>
     <t>a-tag</t>
   </si>
   <si>
     <t>a-project-name</t>
+  </si>
+  <si>
+    <t>a-description</t>
   </si>
 </sst>
 </file>
@@ -1201,13 +1201,13 @@
         <v>44562</v>
       </c>
       <c r="B7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>14</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>12</v>
       </c>
       <c r="E7" s="9">
         <v>2</v>

</xml_diff>